<commit_message>
Add Policy Number and Carrier to bulk upload template for dedup support
</commit_message>
<xml_diff>
--- a/test_customers.xlsx
+++ b/test_customers.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,50 +424,60 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Policy Number</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Carrier</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Policy Type</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Policy Duration (yrs)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Renewal Date</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Premium Change</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Premium Change Reason</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>At-Fault Claims (3yr)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Bundle Status</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Payment Record</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Last Contact</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -481,46 +491,56 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>POL-100001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Progressive</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="E2" t="n">
         <v>1.5</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>2026-07-20</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Increased 25-50%</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>at-fault accident</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="I2" t="n">
         <v>1</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Auto Only</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Occasionally Late</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>3-6 months ago</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Mentioned comparing quotes online</t>
         </is>
@@ -534,46 +554,56 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>POL-100002</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>State Farm</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="E3" t="n">
         <v>8</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Flat</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="I3" t="n">
         <v>0</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Home Only</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Always On Time</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>1-3 months ago</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -583,46 +613,56 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>POL-100003</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GEICO</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="E4" t="n">
         <v>3</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Increased 50%+</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>2 at-fault claims</t>
         </is>
       </c>
-      <c r="G4" t="n">
+      <c r="I4" t="n">
         <v>2</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Auto Only</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Frequently Late</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>6+ months ago</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Very unhappy about rate increase</t>
         </is>
@@ -636,46 +676,56 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>POL-100004</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Allstate</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>Auto + Home</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="E5" t="n">
         <v>12</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>2026-10-03</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Increased 0-10%</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>area risk increase</t>
         </is>
       </c>
-      <c r="G5" t="n">
+      <c r="I5" t="n">
         <v>0</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Auto + Home</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Always On Time</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Within 1 month</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Long-term loyal customer</t>
         </is>
@@ -689,46 +739,56 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>POL-100005</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Progressive</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="E6" t="n">
         <v>0.5</v>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Increased 25-50%</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>at-fault accident</t>
         </is>
       </c>
-      <c r="G6" t="n">
+      <c r="I6" t="n">
         <v>1</v>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Auto Only</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Occasionally Late</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>3-6 months ago</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Asked about switching</t>
         </is>
@@ -742,46 +802,56 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>POL-100006</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Farmers</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>Renters</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="E7" t="n">
         <v>2</v>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Increased 10-25%</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>credit score change</t>
         </is>
       </c>
-      <c r="G7" t="n">
+      <c r="I7" t="n">
         <v>0</v>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Renters Only</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>Always On Time</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>1-3 months ago</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -791,46 +861,56 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>POL-100007</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>State Farm</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="C8" t="n">
+      <c r="E8" t="n">
         <v>5</v>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>2026-11-02</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Flat</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G8" t="n">
+      <c r="I8" t="n">
         <v>0</v>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Auto + Life</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>Always On Time</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>6+ months ago</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>Happy with service</t>
         </is>
@@ -844,46 +924,56 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>POL-100008</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Nationwide</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="E9" t="n">
         <v>15</v>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>2027-01-01</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Decreased</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>loyalty discount</t>
         </is>
       </c>
-      <c r="G9" t="n">
+      <c r="I9" t="n">
         <v>0</v>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Auto + Home</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>Always On Time</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>Within 1 month</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>Referred 2 friends</t>
         </is>
@@ -897,46 +987,56 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>POL-100009</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>GEICO</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="C10" t="n">
+      <c r="E10" t="n">
         <v>1</v>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Increased 50%+</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>DUI conviction</t>
         </is>
       </c>
-      <c r="G10" t="n">
+      <c r="I10" t="n">
         <v>1</v>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Auto Only</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Frequently Late</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>6+ months ago</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>Has court date pending</t>
         </is>
@@ -950,46 +1050,56 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>POL-100010</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Allstate</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
           <t>Auto + Home</t>
         </is>
       </c>
-      <c r="C11" t="n">
+      <c r="E11" t="n">
         <v>7</v>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Increased 10-25%</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>minor traffic violation</t>
         </is>
       </c>
-      <c r="G11" t="n">
+      <c r="I11" t="n">
         <v>0</v>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Auto + Home</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>Always On Time</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>1-3 months ago</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>Recently married</t>
         </is>

</xml_diff>